<commit_message>
v1.9 added Dice roll sounds and audio assets for Countess Spatula and Johnny Dynamite
</commit_message>
<xml_diff>
--- a/.audio_bank_1.2.xlsx
+++ b/.audio_bank_1.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nbs\yay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3355492-EB29-4E7C-B530-2543F55E488D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11760FE-A31A-4EEB-950A-D11BA7FD9685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3720" yWindow="3720" windowWidth="19200" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2582,9 +2582,6 @@
     <t>"Keeping these right here in the studio."</t>
   </si>
   <si>
-    <t>"That's a solid hit! Maybe not top ten, but it'll chart!"</t>
-  </si>
-  <si>
     <t>"A totally tubular score. I'll log it."</t>
   </si>
   <si>
@@ -2597,9 +2594,6 @@
     <t>"We are climbing the charts, baby! Nothing but platinum!"</t>
   </si>
   <si>
-    <t>"Ouch. Dead air. That's the worst sound in radio, folks."</t>
-  </si>
-  <si>
     <t>"Looks like the tape jammed on that one. We're taking a zero."</t>
   </si>
   <si>
@@ -2621,9 +2615,6 @@
     <t>"You're climbing the charts fast, but can you dethrone Donnie the Dial?"</t>
   </si>
   <si>
-    <t>"Nice score! Almost as nice as the upholstery at Pete's Waterbeds!"</t>
-  </si>
-  <si>
     <t>"The competition is fierce today! Just like the prices at Maple Grove Discount Grocery!"</t>
   </si>
   <si>
@@ -2633,15 +2624,9 @@
     <t>"Five of a kind! That is totally tubular! Give this player a prize!"</t>
   </si>
   <si>
-    <t>"Dead air on your end. That's gonna cost you in the ratings."</t>
-  </si>
-  <si>
     <t>"Ouch, took a zero. That's like forgetting to press record on the mixtape."</t>
   </si>
   <si>
-    <t>"Nothing but static for you on that category. Tough break."</t>
-  </si>
-  <si>
     <t>"Donnie's dominating the airwaves! No one can touch this signal!"</t>
   </si>
   <si>
@@ -2675,15 +2660,9 @@
     <t>"Blowing past you on the charts! See you in the rearview mirror!"</t>
   </si>
   <si>
-    <t>"Back to number one! And speaking of numbers, dial 555-0199 for Maple Grove Plumbing!"</t>
-  </si>
-  <si>
     <t>"Donnie takes the win! Thanks for tuning in, and remember to keep your feet on the ground!"</t>
   </si>
   <si>
-    <t>"We finish at the top of the charts! This victory is brought to you by Pete's Waterbeds!"</t>
-  </si>
-  <si>
     <t>"Signing off as the champion! Catch you on the flip side, baby!"</t>
   </si>
   <si>
@@ -2726,15 +2705,9 @@
     <t>"Just paying the bills, folks. Just like our sponsors at the 24-Hour Discount Dental Clinic."</t>
   </si>
   <si>
-    <t>"That's a hit! Not a smash hit, but it'll get radio play!"</t>
-  </si>
-  <si>
     <t>"Points on the board, brought to you by the Maple Grove Discount Toupee Outlet!"</t>
   </si>
   <si>
-    <t>"We'll spin that track. Good points."</t>
-  </si>
-  <si>
     <t>"A YAY! That's a diamond record! And speaking of diamonds, visit the Maple Grove Jewelers and Discount Mattress Center!"</t>
   </si>
   <si>
@@ -2925,6 +2898,33 @@
   </si>
   <si>
     <t>"This is the darkest timeline! I concede defeat! Now leave my lair before I throw a sponge at you!"</t>
+  </si>
+  <si>
+    <t>You’re locked in and rocking with the boss of the airwaves! Don't touch those dice.</t>
+  </si>
+  <si>
+    <t>You're cruising with the captain of the airwaves! Smooth sailing and rockin' rolls all night long.</t>
+  </si>
+  <si>
+    <t>Ouch, scratch! That's worse than dead air on radio</t>
+  </si>
+  <si>
+    <t>It's the bottom of the hour … but you're flyin' high with that score</t>
+  </si>
+  <si>
+    <t>It's bumper to bumper out there. No movement at all … just like your last scratch!</t>
+  </si>
+  <si>
+    <t>This is your drive-time jam to get you through the slam… Was taking a zero part of your plan?</t>
+  </si>
+  <si>
+    <t>We've got the weather, the traffic, and the tunes to make your rolls a total breeze!</t>
+  </si>
+  <si>
+    <t>A win for me … and you the listener! 60 minutes of commercial free music … right after this 15 minute break.</t>
+  </si>
+  <si>
+    <t>We are keeping the music flowing and the good times rolling, brought to you by Gary's Gently Used Mayonnaise.</t>
   </si>
 </sst>
 </file>
@@ -3319,8 +3319,7 @@
   <cols>
     <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -3351,14 +3350,14 @@
       <c r="I1" s="1" t="s">
         <v>673</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>807</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>814</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>276</v>
@@ -3421,13 +3420,13 @@
       <c r="I2" t="s">
         <v>799</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>815</v>
       </c>
+      <c r="L2" s="3"/>
       <c r="M2" s="1" t="s">
         <v>483</v>
       </c>
@@ -3458,13 +3457,13 @@
       <c r="I3" t="s">
         <v>803</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" t="s">
+        <v>807</v>
+      </c>
       <c r="K3" t="s">
-        <v>807</v>
-      </c>
-      <c r="L3" t="s">
         <v>805</v>
       </c>
+      <c r="L3" s="3"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="3"/>
@@ -3497,7 +3496,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:24" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -3516,9 +3515,6 @@
       </c>
       <c r="H5" s="2" t="s">
         <v>473</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>864</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>474</v>
@@ -3552,14 +3548,14 @@
       <c r="I6" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="2" t="s">
+        <v>857</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>865</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>879</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>280</v>
@@ -3605,14 +3601,14 @@
       <c r="I7" s="2" t="s">
         <v>677</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="2" t="s">
+        <v>858</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>871</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>816</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>880</v>
       </c>
       <c r="N7" s="2" t="s">
         <v>283</v>
@@ -3658,14 +3654,14 @@
       <c r="I8" s="2" t="s">
         <v>679</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>872</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>817</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>881</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>286</v>
@@ -3683,7 +3679,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="238.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:24" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -3711,14 +3707,14 @@
       <c r="I9" s="2" t="s">
         <v>681</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="L9" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>866</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>882</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>289</v>
@@ -3736,7 +3732,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="196.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:24" ht="238.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
@@ -3764,14 +3760,14 @@
       <c r="I10" s="2" t="s">
         <v>683</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="2" t="s">
+        <v>859</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="L10" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>818</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>883</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>292</v>
@@ -3817,14 +3813,14 @@
       <c r="I11" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="2" t="s">
+        <v>818</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="L11" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>867</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>884</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>295</v>
@@ -3842,7 +3838,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:24" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
@@ -3870,14 +3866,14 @@
       <c r="I12" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>876</v>
+      </c>
+      <c r="L12" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>868</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>885</v>
       </c>
       <c r="N12" s="2" t="s">
         <v>297</v>
@@ -3895,7 +3891,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:24" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
@@ -3923,14 +3919,14 @@
       <c r="I13" s="2" t="s">
         <v>689</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="2" t="s">
+        <v>861</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>877</v>
+      </c>
+      <c r="L13" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>869</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>886</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>300</v>
@@ -3976,14 +3972,14 @@
       <c r="I14" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="2" t="s">
+        <v>862</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="L14" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>819</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>887</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>302</v>
@@ -4029,14 +4025,14 @@
       <c r="I15" s="2" t="s">
         <v>693</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="J15" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>879</v>
+      </c>
+      <c r="L15" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>870</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>888</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>305</v>
@@ -4082,14 +4078,14 @@
       <c r="I16" s="2" t="s">
         <v>695</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="J16" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>880</v>
+      </c>
+      <c r="L16" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>871</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>889</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>308</v>
@@ -4135,14 +4131,14 @@
       <c r="I17" s="2" t="s">
         <v>697</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="2" t="s">
+        <v>864</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="L17" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>820</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>890</v>
       </c>
       <c r="N17" s="2" t="s">
         <v>311</v>
@@ -4188,14 +4184,14 @@
       <c r="I18" s="2" t="s">
         <v>699</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="L18" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>821</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>891</v>
       </c>
       <c r="N18" s="2" t="s">
         <v>314</v>
@@ -4241,14 +4237,14 @@
       <c r="I19" s="2" t="s">
         <v>701</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J19" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="L19" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>822</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>892</v>
       </c>
       <c r="N19" s="2" t="s">
         <v>317</v>
@@ -4294,14 +4290,14 @@
       <c r="I20" s="2" t="s">
         <v>703</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="J20" s="2" t="s">
+        <v>822</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>884</v>
+      </c>
+      <c r="L20" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>823</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>893</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>320</v>
@@ -4347,14 +4343,14 @@
       <c r="I21" s="2" t="s">
         <v>705</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="J21" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>885</v>
+      </c>
+      <c r="L21" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>824</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>894</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>323</v>
@@ -4400,14 +4396,14 @@
       <c r="I22" s="2" t="s">
         <v>707</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="J22" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="L22" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>895</v>
       </c>
       <c r="N22" s="2" t="s">
         <v>326</v>
@@ -4425,7 +4421,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
@@ -4453,14 +4449,14 @@
       <c r="I23" s="2" t="s">
         <v>709</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="2" t="s">
+        <v>937</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="L23" t="s">
         <v>27</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>896</v>
       </c>
       <c r="N23" s="2" t="s">
         <v>329</v>
@@ -4506,14 +4502,14 @@
       <c r="I24" s="2" t="s">
         <v>711</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="L24" t="s">
         <v>28</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>872</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>897</v>
       </c>
       <c r="N24" s="2" t="s">
         <v>332</v>
@@ -4531,7 +4527,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
@@ -4559,14 +4555,14 @@
       <c r="I25" s="2" t="s">
         <v>713</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="2" t="s">
+        <v>865</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="L25" t="s">
         <v>30</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>873</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>898</v>
       </c>
       <c r="N25" s="2" t="s">
         <v>335</v>
@@ -4584,7 +4580,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>26</v>
       </c>
@@ -4612,14 +4608,14 @@
       <c r="I26" s="2" t="s">
         <v>715</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="2" t="s">
+        <v>931</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>890</v>
+      </c>
+      <c r="L26" t="s">
         <v>31</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>874</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>899</v>
       </c>
       <c r="N26" s="2" t="s">
         <v>338</v>
@@ -4637,7 +4633,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
@@ -4665,14 +4661,14 @@
       <c r="I27" s="2" t="s">
         <v>717</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="L27" t="s">
         <v>32</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>875</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>900</v>
       </c>
       <c r="N27" s="2" t="s">
         <v>341</v>
@@ -4690,7 +4686,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:18" ht="196.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
@@ -4718,14 +4714,14 @@
       <c r="I28" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>892</v>
+      </c>
+      <c r="L28" t="s">
         <v>29</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>827</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>901</v>
       </c>
       <c r="N28" s="2" t="s">
         <v>344</v>
@@ -4771,14 +4767,14 @@
       <c r="I29" s="2" t="s">
         <v>721</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>893</v>
+      </c>
+      <c r="L29" t="s">
         <v>34</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>828</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>902</v>
       </c>
       <c r="N29" s="2" t="s">
         <v>347</v>
@@ -4824,14 +4820,14 @@
       <c r="I30" s="2" t="s">
         <v>723</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="L30" t="s">
         <v>36</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>829</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>903</v>
       </c>
       <c r="N30" s="2" t="s">
         <v>350</v>
@@ -4877,14 +4873,14 @@
       <c r="I31" s="2" t="s">
         <v>725</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="L31" t="s">
         <v>35</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>904</v>
       </c>
       <c r="N31" s="2" t="s">
         <v>353</v>
@@ -4930,14 +4926,14 @@
       <c r="I32" s="2" t="s">
         <v>727</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="2" t="s">
+        <v>933</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="L32" t="s">
         <v>38</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>831</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>905</v>
       </c>
       <c r="N32" s="2" t="s">
         <v>356</v>
@@ -4983,14 +4979,14 @@
       <c r="I33" s="2" t="s">
         <v>729</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J33" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>897</v>
+      </c>
+      <c r="L33" t="s">
         <v>39</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>832</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>906</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>359</v>
@@ -5036,14 +5032,14 @@
       <c r="I34" s="2" t="s">
         <v>731</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J34" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="L34" t="s">
         <v>40</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>833</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>907</v>
       </c>
       <c r="N34" s="2" t="s">
         <v>362</v>
@@ -5089,14 +5085,14 @@
       <c r="I35" s="2" t="s">
         <v>733</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J35" s="2" t="s">
+        <v>831</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="L35" t="s">
         <v>42</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>876</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>908</v>
       </c>
       <c r="N35" s="2" t="s">
         <v>365</v>
@@ -5114,7 +5110,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="224.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:18" ht="238.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
         <v>41</v>
       </c>
@@ -5142,14 +5138,14 @@
       <c r="I36" s="2" t="s">
         <v>735</v>
       </c>
-      <c r="J36" t="s">
+      <c r="J36" s="2" t="s">
+        <v>867</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>900</v>
+      </c>
+      <c r="L36" t="s">
         <v>43</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>877</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>909</v>
       </c>
       <c r="N36" s="2" t="s">
         <v>368</v>
@@ -5167,7 +5163,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>44</v>
       </c>
@@ -5195,14 +5191,14 @@
       <c r="I37" s="2" t="s">
         <v>737</v>
       </c>
-      <c r="J37" t="s">
+      <c r="J37" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>901</v>
+      </c>
+      <c r="L37" t="s">
         <v>45</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>834</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>910</v>
       </c>
       <c r="N37" s="2" t="s">
         <v>371</v>
@@ -5248,14 +5244,14 @@
       <c r="I38" s="2" t="s">
         <v>739</v>
       </c>
-      <c r="J38" t="s">
+      <c r="J38" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>902</v>
+      </c>
+      <c r="L38" t="s">
         <v>47</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>835</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>911</v>
       </c>
       <c r="N38" s="2" t="s">
         <v>374</v>
@@ -5301,14 +5297,14 @@
       <c r="I39" s="2" t="s">
         <v>741</v>
       </c>
-      <c r="J39" t="s">
+      <c r="J39" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="L39" t="s">
         <v>46</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>836</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>912</v>
       </c>
       <c r="N39" s="2" t="s">
         <v>377</v>
@@ -5354,14 +5350,14 @@
       <c r="I40" s="2" t="s">
         <v>743</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>904</v>
+      </c>
+      <c r="L40" t="s">
         <v>49</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>837</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>913</v>
       </c>
       <c r="N40" s="2" t="s">
         <v>380</v>
@@ -5407,14 +5403,14 @@
       <c r="I41" s="2" t="s">
         <v>745</v>
       </c>
-      <c r="J41" t="s">
+      <c r="J41" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>905</v>
+      </c>
+      <c r="L41" t="s">
         <v>50</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>838</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>914</v>
       </c>
       <c r="N41" s="2" t="s">
         <v>383</v>
@@ -5432,7 +5428,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
         <v>48</v>
       </c>
@@ -5460,14 +5456,14 @@
       <c r="I42" s="2" t="s">
         <v>747</v>
       </c>
-      <c r="J42" t="s">
+      <c r="J42" s="2" t="s">
+        <v>934</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>906</v>
+      </c>
+      <c r="L42" t="s">
         <v>51</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>839</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>915</v>
       </c>
       <c r="N42" s="2" t="s">
         <v>386</v>
@@ -5485,7 +5481,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:18" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
         <v>48</v>
       </c>
@@ -5513,14 +5509,14 @@
       <c r="I43" s="2" t="s">
         <v>749</v>
       </c>
-      <c r="J43" t="s">
+      <c r="J43" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>907</v>
+      </c>
+      <c r="L43" t="s">
         <v>52</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>840</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>916</v>
       </c>
       <c r="N43" s="2" t="s">
         <v>389</v>
@@ -5566,14 +5562,14 @@
       <c r="I44" s="2" t="s">
         <v>751</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>908</v>
+      </c>
+      <c r="L44" t="s">
         <v>54</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>841</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>917</v>
       </c>
       <c r="N44" s="2" t="s">
         <v>392</v>
@@ -5619,14 +5615,14 @@
       <c r="I45" s="2" t="s">
         <v>753</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J45" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>909</v>
+      </c>
+      <c r="L45" t="s">
         <v>55</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>842</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>918</v>
       </c>
       <c r="N45" s="2" t="s">
         <v>395</v>
@@ -5644,7 +5640,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:18" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
         <v>56</v>
       </c>
@@ -5672,14 +5668,14 @@
       <c r="I46" s="2" t="s">
         <v>755</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J46" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>910</v>
+      </c>
+      <c r="L46" t="s">
         <v>57</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>843</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>919</v>
       </c>
       <c r="N46" s="2" t="s">
         <v>398</v>
@@ -5725,14 +5721,14 @@
       <c r="I47" s="2" t="s">
         <v>757</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J47" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>911</v>
+      </c>
+      <c r="L47" t="s">
         <v>58</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>844</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>920</v>
       </c>
       <c r="N47" s="2" t="s">
         <v>401</v>
@@ -5750,7 +5746,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:18" ht="196.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
         <v>56</v>
       </c>
@@ -5778,14 +5774,14 @@
       <c r="I48" s="2" t="s">
         <v>759</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="2" t="s">
+        <v>936</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="L48" t="s">
         <v>59</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>845</v>
-      </c>
-      <c r="L48" s="2" t="s">
-        <v>921</v>
       </c>
       <c r="N48" s="2" t="s">
         <v>404</v>
@@ -5831,14 +5827,14 @@
       <c r="I49" s="2" t="s">
         <v>761</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J49" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="L49" t="s">
         <v>61</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>846</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>922</v>
       </c>
       <c r="N49" s="2" t="s">
         <v>407</v>
@@ -5884,14 +5880,14 @@
       <c r="I50" s="2" t="s">
         <v>763</v>
       </c>
-      <c r="J50" t="s">
+      <c r="J50" s="2" t="s">
+        <v>841</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>914</v>
+      </c>
+      <c r="L50" t="s">
         <v>62</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>847</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>923</v>
       </c>
       <c r="N50" s="2" t="s">
         <v>410</v>
@@ -5909,7 +5905,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:18" ht="154.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="4" t="s">
         <v>60</v>
       </c>
@@ -5937,14 +5933,14 @@
       <c r="I51" s="2" t="s">
         <v>765</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J51" s="2" t="s">
+        <v>842</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>915</v>
+      </c>
+      <c r="L51" t="s">
         <v>63</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>848</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>924</v>
       </c>
       <c r="N51" s="2" t="s">
         <v>413</v>
@@ -5990,14 +5986,14 @@
       <c r="I52" s="2" t="s">
         <v>767</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J52" s="2" t="s">
+        <v>843</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="L52" t="s">
         <v>65</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>849</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>925</v>
       </c>
       <c r="N52" s="2" t="s">
         <v>416</v>
@@ -6015,7 +6011,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="168.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:18" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="4" t="s">
         <v>64</v>
       </c>
@@ -6043,14 +6039,14 @@
       <c r="I53" s="2" t="s">
         <v>769</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J53" s="2" t="s">
+        <v>844</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="L53" t="s">
         <v>66</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>850</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>926</v>
       </c>
       <c r="N53" s="2" t="s">
         <v>419</v>
@@ -6096,14 +6092,14 @@
       <c r="I54" s="2" t="s">
         <v>771</v>
       </c>
-      <c r="J54" t="s">
+      <c r="J54" s="2" t="s">
+        <v>845</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>918</v>
+      </c>
+      <c r="L54" t="s">
         <v>67</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>851</v>
-      </c>
-      <c r="L54" s="2" t="s">
-        <v>927</v>
       </c>
       <c r="N54" s="2" t="s">
         <v>422</v>
@@ -6149,14 +6145,14 @@
       <c r="I55" s="2" t="s">
         <v>773</v>
       </c>
-      <c r="J55" t="s">
+      <c r="J55" s="2" t="s">
+        <v>846</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="L55" t="s">
         <v>69</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>852</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>928</v>
       </c>
       <c r="N55" s="2" t="s">
         <v>425</v>
@@ -6174,7 +6170,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="126.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:18" ht="140.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
         <v>68</v>
       </c>
@@ -6202,14 +6198,14 @@
       <c r="I56" s="2" t="s">
         <v>775</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J56" s="2" t="s">
+        <v>847</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>920</v>
+      </c>
+      <c r="L56" t="s">
         <v>70</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>853</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>929</v>
       </c>
       <c r="N56" s="2" t="s">
         <v>428</v>
@@ -6255,14 +6251,14 @@
       <c r="I57" s="2" t="s">
         <v>777</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J57" s="2" t="s">
+        <v>848</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>921</v>
+      </c>
+      <c r="L57" t="s">
         <v>71</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>854</v>
-      </c>
-      <c r="L57" s="2" t="s">
-        <v>930</v>
       </c>
       <c r="N57" s="2" t="s">
         <v>431</v>
@@ -6308,14 +6304,14 @@
       <c r="I58" s="2" t="s">
         <v>779</v>
       </c>
-      <c r="J58" t="s">
+      <c r="J58" s="2" t="s">
+        <v>849</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="L58" t="s">
         <v>73</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>855</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>931</v>
       </c>
       <c r="N58" s="2" t="s">
         <v>434</v>
@@ -6361,14 +6357,14 @@
       <c r="I59" s="2" t="s">
         <v>781</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J59" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>923</v>
+      </c>
+      <c r="L59" t="s">
         <v>74</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>856</v>
-      </c>
-      <c r="L59" s="2" t="s">
-        <v>932</v>
       </c>
       <c r="N59" s="2" t="s">
         <v>437</v>
@@ -6386,7 +6382,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="182.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:18" ht="238.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
         <v>72</v>
       </c>
@@ -6414,14 +6410,14 @@
       <c r="I60" s="2" t="s">
         <v>783</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J60" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>924</v>
+      </c>
+      <c r="L60" t="s">
         <v>75</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>857</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>933</v>
       </c>
       <c r="N60" s="2" t="s">
         <v>439</v>
@@ -6467,14 +6463,14 @@
       <c r="I61" s="2" t="s">
         <v>785</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J61" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>925</v>
+      </c>
+      <c r="L61" t="s">
         <v>77</v>
-      </c>
-      <c r="K61" s="2" t="s">
-        <v>858</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>934</v>
       </c>
       <c r="N61" s="2" t="s">
         <v>442</v>
@@ -6492,7 +6488,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="210.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:18" ht="224.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
         <v>76</v>
       </c>
@@ -6520,14 +6516,14 @@
       <c r="I62" s="2" t="s">
         <v>787</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J62" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>926</v>
+      </c>
+      <c r="L62" t="s">
         <v>78</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>859</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>935</v>
       </c>
       <c r="N62" s="2" t="s">
         <v>445</v>
@@ -6573,14 +6569,14 @@
       <c r="I63" s="2" t="s">
         <v>789</v>
       </c>
-      <c r="J63" t="s">
+      <c r="J63" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="L63" t="s">
         <v>79</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>878</v>
-      </c>
-      <c r="L63" s="2" t="s">
-        <v>936</v>
       </c>
       <c r="N63" s="2" t="s">
         <v>448</v>
@@ -6626,14 +6622,14 @@
       <c r="I64" s="2" t="s">
         <v>791</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J64" s="2" t="s">
+        <v>869</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>928</v>
+      </c>
+      <c r="L64" t="s">
         <v>81</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>860</v>
-      </c>
-      <c r="L64" s="2" t="s">
-        <v>937</v>
       </c>
       <c r="N64" s="2" t="s">
         <v>451</v>
@@ -6679,14 +6675,14 @@
       <c r="I65" s="2" t="s">
         <v>793</v>
       </c>
-      <c r="J65" t="s">
+      <c r="J65" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="L65" t="s">
         <v>82</v>
-      </c>
-      <c r="K65" s="2" t="s">
-        <v>861</v>
-      </c>
-      <c r="L65" s="2" t="s">
-        <v>938</v>
       </c>
       <c r="N65" s="2" t="s">
         <v>454</v>
@@ -6732,14 +6728,14 @@
       <c r="I66" s="2" t="s">
         <v>795</v>
       </c>
-      <c r="J66" t="s">
+      <c r="J66" s="2" t="s">
+        <v>854</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="L66" t="s">
         <v>83</v>
-      </c>
-      <c r="K66" s="2" t="s">
-        <v>862</v>
-      </c>
-      <c r="L66" s="2" t="s">
-        <v>939</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>457</v>
@@ -6785,12 +6781,14 @@
       <c r="I67" s="2" t="s">
         <v>797</v>
       </c>
-      <c r="J67" t="s">
+      <c r="J67" s="2" t="s">
+        <v>855</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>856</v>
+      </c>
+      <c r="L67" t="s">
         <v>84</v>
-      </c>
-      <c r="K67" s="2"/>
-      <c r="L67" s="2" t="s">
-        <v>863</v>
       </c>
       <c r="M67" s="2" t="s">
         <v>460</v>

</xml_diff>